<commit_message>
Fixes accross all different users
</commit_message>
<xml_diff>
--- a/test.xlsx
+++ b/test.xlsx
@@ -375,19 +375,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:E3"/>
   <cols>
     <col min="1" max="1" width="20.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
     <col min="3" max="3" width="10.83203125" customWidth="1"/>
     <col min="4" max="4" width="12.83203125" customWidth="1"/>
     <col min="5" max="5" width="10.83203125" customWidth="1"/>
-    <col min="6" max="6" width="12.83203125" customWidth="1"/>
-    <col min="7" max="7" width="10.83203125" customWidth="1"/>
-    <col min="8" max="8" width="12.83203125" customWidth="1"/>
-    <col min="9" max="9" width="10.83203125" customWidth="1"/>
-    <col min="10" max="10" width="12.83203125" customWidth="1"/>
-    <col min="11" max="11" width="10.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -395,19 +389,10 @@
         <v>Fullname</v>
       </c>
       <c r="B1" t="str">
-        <v>ENGLISH LANGUAGE</v>
+        <v>AGRICULTURAL SCIENCE</v>
       </c>
       <c r="D1" t="str">
-        <v>CHEMISTRY</v>
-      </c>
-      <c r="F1" t="str">
-        <v>PHYSICS</v>
-      </c>
-      <c r="H1" t="str">
         <v>MATHEMATICS</v>
-      </c>
-      <c r="J1" t="str">
-        <v>BIOLOGY</v>
       </c>
     </row>
     <row r="2">
@@ -426,28 +411,10 @@
       <c r="E2" t="str">
         <v>Exam</v>
       </c>
-      <c r="F2" t="str">
-        <v>CA</v>
-      </c>
-      <c r="G2" t="str">
-        <v>Exam</v>
-      </c>
-      <c r="H2" t="str">
-        <v>CA</v>
-      </c>
-      <c r="I2" t="str">
-        <v>Exam</v>
-      </c>
-      <c r="J2" t="str">
-        <v>CA</v>
-      </c>
-      <c r="K2" t="str">
-        <v>Exam</v>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>YEYE ADE</v>
+        <v>WEDE SAFIU</v>
       </c>
       <c r="B3" t="str">
         <v/>
@@ -461,70 +428,14 @@
       <c r="E3" t="str">
         <v/>
       </c>
-      <c r="F3" t="str">
-        <v/>
-      </c>
-      <c r="G3" t="str">
-        <v/>
-      </c>
-      <c r="H3" t="str">
-        <v/>
-      </c>
-      <c r="I3" t="str">
-        <v/>
-      </c>
-      <c r="J3" t="str">
-        <v/>
-      </c>
-      <c r="K3" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>OLALADE ASAKE</v>
-      </c>
-      <c r="B4" t="str">
-        <v/>
-      </c>
-      <c r="C4" t="str">
-        <v/>
-      </c>
-      <c r="D4" t="str">
-        <v/>
-      </c>
-      <c r="E4" t="str">
-        <v/>
-      </c>
-      <c r="F4" t="str">
-        <v/>
-      </c>
-      <c r="G4" t="str">
-        <v/>
-      </c>
-      <c r="H4" t="str">
-        <v/>
-      </c>
-      <c r="I4" t="str">
-        <v/>
-      </c>
-      <c r="J4" t="str">
-        <v/>
-      </c>
-      <c r="K4" t="str">
-        <v/>
-      </c>
     </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="2">
     <mergeCell ref="B1:C1"/>
     <mergeCell ref="D1:E1"/>
-    <mergeCell ref="F1:G1"/>
-    <mergeCell ref="H1:I1"/>
-    <mergeCell ref="J1:K1"/>
   </mergeCells>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>